<commit_message>
Update macroeconomic indicators documentation with revised Excel file
- Updated the macroeconomic indicators Excel file to reflect recent changes in data entries and classifications.
- Ensured the documentation aligns with the latest dataset adjustments for improved accuracy and usability.
</commit_message>
<xml_diff>
--- a/docs/智能投顾数据.xlsx
+++ b/docs/智能投顾数据.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30460" windowHeight="18180"/>
+    <workbookView windowHeight="18180" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="境内宏观" sheetId="1" r:id="rId1"/>
@@ -14,8 +14,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">境内宏观!$A$1:$J$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">境外宏观!$A$1:$I$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">大类资产!$A$1:$J$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">境外宏观!$A$1:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">大类资产!$A$1:$J$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">行情展示!$A$1:$J$21</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1492" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1473" uniqueCount="337">
   <si>
     <t>指标代码</t>
   </si>
@@ -861,6 +861,18 @@
   </si>
   <si>
     <t>E1000174</t>
+  </si>
+  <si>
+    <t>另类资产</t>
+  </si>
+  <si>
+    <t>南华商品指数</t>
+  </si>
+  <si>
+    <t>NHCI</t>
+  </si>
+  <si>
+    <t>商品主腿</t>
   </si>
   <si>
     <t>Ticker</t>
@@ -1547,152 +1559,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="5">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1704,6 +1716,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2062,10 +2077,10 @@
     <col min="6" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="35" customWidth="1"/>
+    <col min="10" max="10" width="20.6953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17" spans="1:10">
+    <row r="1" ht="17" customHeight="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3289,8 +3304,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -3298,10 +3313,9 @@
     <col min="4" max="5" width="8" customWidth="1"/>
     <col min="6" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17" spans="1:9">
+    <row r="1" ht="17" customHeight="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3326,11 +3340,8 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -3355,11 +3366,8 @@
       <c r="H2" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
@@ -3384,11 +3392,8 @@
       <c r="H3" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="I3" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -3413,11 +3418,8 @@
       <c r="H4" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
@@ -3442,11 +3444,8 @@
       <c r="H5" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -3471,11 +3470,8 @@
       <c r="H6" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="I6" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
@@ -3500,11 +3496,8 @@
       <c r="H7" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="I7" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -3529,11 +3522,8 @@
       <c r="H8" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="I8" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
@@ -3558,11 +3548,8 @@
       <c r="H9" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="I9" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -3587,11 +3574,8 @@
       <c r="H10" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="I10" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" s="3" t="s">
         <v>10</v>
       </c>
@@ -3616,11 +3600,8 @@
       <c r="H11" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="I11" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -3645,11 +3626,8 @@
       <c r="H12" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="I12" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" s="3" t="s">
         <v>10</v>
       </c>
@@ -3674,11 +3652,8 @@
       <c r="H13" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="I13" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
@@ -3703,11 +3678,8 @@
       <c r="H14" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" s="3" t="s">
         <v>10</v>
       </c>
@@ -3732,11 +3704,8 @@
       <c r="H15" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="I15" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" s="2" t="s">
         <v>10</v>
       </c>
@@ -3761,11 +3730,8 @@
       <c r="H16" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" s="3" t="s">
         <v>10</v>
       </c>
@@ -3790,11 +3756,8 @@
       <c r="H17" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I17" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" s="2" t="s">
         <v>10</v>
       </c>
@@ -3819,11 +3782,8 @@
       <c r="H18" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="I18" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" s="3" t="s">
         <v>10</v>
       </c>
@@ -3848,11 +3808,8 @@
       <c r="H19" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="I19" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" s="2" t="s">
         <v>10</v>
       </c>
@@ -3877,11 +3834,8 @@
       <c r="H20" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="I20" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" s="3" t="s">
         <v>10</v>
       </c>
@@ -3906,11 +3860,8 @@
       <c r="H21" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="I21" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" s="2" t="s">
         <v>10</v>
       </c>
@@ -3935,11 +3886,8 @@
       <c r="H22" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="I22" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" s="3" t="s">
         <v>10</v>
       </c>
@@ -3964,11 +3912,8 @@
       <c r="H23" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="I23" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" s="2" t="s">
         <v>10</v>
       </c>
@@ -3993,11 +3938,8 @@
       <c r="H24" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="I24" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" s="3" t="s">
         <v>10</v>
       </c>
@@ -4022,12 +3964,9 @@
       <c r="H25" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="I25" s="3" t="s">
-        <v>10</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:I25" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H25" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4038,7 +3977,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -4051,7 +3990,7 @@
     <col min="10" max="10" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17" spans="1:10">
+    <row r="1" ht="17" customHeight="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>119</v>
       </c>
@@ -6227,8 +6166,32 @@
         <v>76</v>
       </c>
     </row>
+    <row r="69" spans="1:10">
+      <c r="A69" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B69" s="2"/>
+      <c r="C69" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="D69" s="2"/>
+      <c r="E69" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="F69" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="G69" s="5"/>
+      <c r="H69" s="2"/>
+      <c r="I69" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>278</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:J68" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:J69" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6251,15 +6214,15 @@
     <col min="10" max="10" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17" spans="1:10">
+    <row r="1" ht="17" customHeight="1" spans="1:10">
       <c r="A1" s="1" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>119</v>
@@ -6285,16 +6248,16 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>10</v>
@@ -6306,7 +6269,7 @@
         <v>10</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>10</v>
@@ -6317,16 +6280,16 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="3" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>280</v>
-      </c>
       <c r="D3" s="3" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>10</v>
@@ -6338,7 +6301,7 @@
         <v>10</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>10</v>
@@ -6349,17 +6312,17 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>281</v>
-      </c>
       <c r="E4" s="2" t="s">
         <v>10</v>
       </c>
@@ -6370,7 +6333,7 @@
         <v>10</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>10</v>
@@ -6381,16 +6344,16 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="3" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>10</v>
@@ -6402,7 +6365,7 @@
         <v>10</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>10</v>
@@ -6413,16 +6376,16 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="2" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>10</v>
@@ -6434,7 +6397,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>10</v>
@@ -6445,16 +6408,16 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="3" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>10</v>
@@ -6466,7 +6429,7 @@
         <v>10</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>10</v>
@@ -6477,16 +6440,16 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="2" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>129</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>10</v>
@@ -6498,7 +6461,7 @@
         <v>10</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>10</v>
@@ -6509,16 +6472,16 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="3" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>10</v>
@@ -6530,7 +6493,7 @@
         <v>10</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>10</v>
@@ -6544,13 +6507,13 @@
         <v>204</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>10</v>
@@ -6562,7 +6525,7 @@
         <v>10</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>204</v>
@@ -6573,16 +6536,16 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="3" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>301</v>
-      </c>
       <c r="D11" s="3" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>10</v>
@@ -6594,7 +6557,7 @@
         <v>10</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>10</v>
@@ -6605,16 +6568,16 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="2" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>10</v>
@@ -6626,7 +6589,7 @@
         <v>10</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>10</v>
@@ -6637,16 +6600,16 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="3" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>10</v>
@@ -6658,7 +6621,7 @@
         <v>10</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>10</v>
@@ -6669,7 +6632,7 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="2" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>136</v>
@@ -6701,10 +6664,10 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="3" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>10</v>
@@ -6722,7 +6685,7 @@
         <v>10</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>10</v>
@@ -6733,10 +6696,10 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="2" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>10</v>
@@ -6754,7 +6717,7 @@
         <v>10</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>10</v>
@@ -6765,10 +6728,10 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="3" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>10</v>
@@ -6786,7 +6749,7 @@
         <v>10</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>10</v>
@@ -6797,10 +6760,10 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="2" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>10</v>
@@ -6818,7 +6781,7 @@
         <v>10</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>139</v>
@@ -6829,16 +6792,16 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="3" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>10</v>
@@ -6850,7 +6813,7 @@
         <v>10</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>255</v>
@@ -6861,16 +6824,16 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="2" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>10</v>
@@ -6882,7 +6845,7 @@
         <v>10</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>10</v>
@@ -6893,16 +6856,16 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="3" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>10</v>
@@ -6914,7 +6877,7 @@
         <v>10</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>10</v>

</xml_diff>